<commit_message>
UI Improvements, example questions, images, progress indicator
</commit_message>
<xml_diff>
--- a/Foundation Skills Spreadsheet.xlsx
+++ b/Foundation Skills Spreadsheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29905"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{482F4520-8E45-476B-A9A2-D37BC42754E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41132264-EEA7-4D09-952D-2A269F6AA9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="103">
   <si>
     <t>Maths Skill</t>
   </si>
@@ -127,6 +127,9 @@
     <t>Simplifying Fractions</t>
   </si>
   <si>
+    <t>Irregular and Top Heavy Fractions</t>
+  </si>
+  <si>
     <t>Decimals</t>
   </si>
   <si>
@@ -148,9 +151,6 @@
     <t>Fractions, Decimals and Percentages</t>
   </si>
   <si>
-    <t>Converitng Fractions to Decimals</t>
-  </si>
-  <si>
     <t>Exact Calculations</t>
   </si>
   <si>
@@ -250,16 +250,10 @@
     <t>Volume of a prism</t>
   </si>
   <si>
-    <t>Areas of a Trapezium</t>
-  </si>
-  <si>
     <t>Volume of a Pyramid and Cone</t>
   </si>
   <si>
     <t>Volume of a Prism</t>
-  </si>
-  <si>
-    <t>Areas of Circles</t>
   </si>
   <si>
     <t>Volume of a Sphere</t>
@@ -780,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.85546875" style="2" customWidth="1"/>
@@ -1074,7 +1068,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1085,10 +1079,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1099,13 +1090,10 @@
         <v>4</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D27" t="s">
         <v>29</v>
-      </c>
-      <c r="E27" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1116,10 +1104,13 @@
         <v>4</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" t="s">
         <v>30</v>
-      </c>
-      <c r="D28" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1149,9 +1140,6 @@
       <c r="D30" t="s">
         <v>3</v>
       </c>
-      <c r="E30" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="2" t="s">
@@ -1161,83 +1149,88 @@
         <v>4</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="B32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="7" t="s">
+      <c r="D32" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C32" s="1" t="s">
+      <c r="B33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="1"/>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="D33" s="1"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D37" s="1"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>15</v>
@@ -1249,7 +1242,7 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>15</v>
@@ -1261,7 +1254,7 @@
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>15</v>
@@ -1269,35 +1262,36 @@
       <c r="C40" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D40" t="s">
-        <v>45</v>
-      </c>
+      <c r="D40" s="1"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>3</v>
+        <v>44</v>
+      </c>
+      <c r="D41" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>24</v>
@@ -1308,18 +1302,18 @@
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>4</v>
@@ -1330,21 +1324,18 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D46" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" s="6" t="s">
-        <v>55</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>9</v>
@@ -1357,19 +1348,22 @@
       </c>
     </row>
     <row r="48" spans="1:4">
-      <c r="A48" s="2" t="s">
-        <v>56</v>
+      <c r="A48" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>9</v>
@@ -1380,274 +1374,274 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="D51" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="D52" t="s">
-        <v>59</v>
-      </c>
-      <c r="E52" t="s">
-        <v>17</v>
-      </c>
-      <c r="F52" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="C53" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D53" t="s">
+        <v>59</v>
+      </c>
+      <c r="E53" t="s">
+        <v>17</v>
+      </c>
+      <c r="F53" t="s">
         <v>29</v>
-      </c>
-      <c r="D53" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>61</v>
+        <v>29</v>
+      </c>
+      <c r="D54" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D55" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>3</v>
+        <v>29</v>
+      </c>
+      <c r="D56" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>65</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="7" t="s">
-        <v>69</v>
+      <c r="A60" s="2" t="s">
+        <v>68</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="2" t="s">
-        <v>70</v>
+      <c r="A61" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D62" t="s">
-        <v>59</v>
-      </c>
-      <c r="E62" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D63" s="1" t="s">
         <v>44</v>
       </c>
+      <c r="D63" t="s">
+        <v>59</v>
+      </c>
       <c r="E63" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D64" t="s">
+        <v>73</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E64" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C65" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D65" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>73</v>
+      <c r="C66" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C67" s="1" t="s">
-        <v>74</v>
+      <c r="C67" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="1:7">
       <c r="A68" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D68" t="s">
-        <v>26</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>25</v>
+        <v>3</v>
+      </c>
+      <c r="D69" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>24</v>
@@ -1658,249 +1652,249 @@
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>5</v>
+        <v>26</v>
       </c>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D73" t="s">
         <v>5</v>
-      </c>
-      <c r="E73" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="74" spans="1:7">
       <c r="A74" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="D74" t="s">
-        <v>67</v>
+        <v>5</v>
+      </c>
+      <c r="E74" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="D75" t="s">
-        <v>14</v>
-      </c>
-      <c r="E75" t="s">
-        <v>5</v>
-      </c>
-      <c r="F75" t="s">
-        <v>44</v>
-      </c>
-      <c r="G75" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C76" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D76" t="s">
         <v>14</v>
       </c>
-      <c r="D76" t="s">
-        <v>20</v>
+      <c r="E76" t="s">
+        <v>5</v>
+      </c>
+      <c r="F76" t="s">
+        <v>44</v>
+      </c>
+      <c r="G76" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>88</v>
+      <c r="C77" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D77" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C78" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D78" t="s">
-        <v>67</v>
+      <c r="C78" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>49</v>
+        <v>3</v>
+      </c>
+      <c r="D79" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>91</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>3</v>
+        <v>89</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D85" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
+      </c>
+      <c r="D86" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C87" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4">
+      <c r="A88" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="D87" t="s">
+      <c r="D88" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4">
-      <c r="A88" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="7" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>100</v>
+        <v>16</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>26</v>
+        <v>98</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="7" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>15</v>
@@ -1908,18 +1902,29 @@
       <c r="C91" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D91" t="s">
-        <v>17</v>
-      </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="7" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C92" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D92" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4">
+      <c r="A93" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>